<commit_message>
feat: integrate dual-system analysis and preserve current work state
Include pending implementation, metadata, documentation, reference reports and verification artifacts. Keep raw CSV and DATAC inputs local as requested. Track DAV-25; manual Electron and Excel acceptance remains pending.
</commit_message>
<xml_diff>
--- a/00 Reference Document/config/LAR_TCL metadata.xlsx
+++ b/00 Reference Document/config/LAR_TCL metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29415"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Test_Code\TOV_Final\CheckerProgram_Manoj\metadataV5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Smart Maintanence\TOV1050_Analyzer\00 Reference Document\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B2DEBE-00BA-442D-AA14-8BDAD394A2DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F03C509B-11DF-42A3-852F-647F69A9935C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="180" windowWidth="14355" windowHeight="15210" xr2:uid="{40971268-6843-45A4-929F-390CE8EC23ED}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{40971268-6843-45A4-929F-390CE8EC23ED}"/>
   </bookViews>
   <sheets>
     <sheet name="threshold" sheetId="3" r:id="rId1"/>
@@ -173,7 +173,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,9 +275,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -315,7 +315,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -421,7 +421,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -563,7 +563,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -572,16 +572,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA354EF1-BC8A-4D36-9E77-3C91C8F99CA2}">
   <dimension ref="A1:F89"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" customWidth="1"/>
-    <col min="6" max="6" width="37.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="9.1796875" customWidth="1"/>
+    <col min="6" max="6" width="37.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -601,7 +601,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -618,7 +618,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -638,7 +638,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -658,7 +658,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -675,7 +675,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -692,7 +692,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -712,7 +712,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -732,7 +732,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -749,7 +749,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -766,7 +766,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -786,7 +786,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -806,7 +806,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -823,7 +823,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -840,7 +840,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -860,7 +860,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -880,7 +880,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -897,7 +897,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -914,7 +914,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -934,7 +934,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -951,7 +951,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -971,7 +971,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -988,7 +988,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -1025,7 +1025,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>13</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>6</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>6</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -1096,7 +1096,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -1113,7 +1113,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>6</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>6</v>
       </c>
@@ -1150,7 +1150,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>6</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>6</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>6</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>6</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>6</v>
       </c>
@@ -1264,7 +1264,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>6</v>
       </c>
@@ -1284,7 +1284,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -1318,7 +1318,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -1412,7 +1412,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -1432,7 +1432,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -1472,7 +1472,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="7" t="s">
         <v>28</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="7" t="s">
         <v>28</v>
       </c>
@@ -1526,7 +1526,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="7" t="s">
         <v>28</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="7" t="s">
         <v>28</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="7" t="s">
         <v>28</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="7" t="s">
         <v>28</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="7" t="s">
         <v>28</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="7" t="s">
         <v>28</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="7" t="s">
         <v>28</v>
       </c>
@@ -1655,7 +1655,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="7" t="s">
         <v>28</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="7" t="s">
         <v>28</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="7" t="s">
         <v>28</v>
       </c>
@@ -1713,7 +1713,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
         <v>28</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
         <v>28</v>
       </c>
@@ -1751,7 +1751,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="7" t="s">
         <v>28</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
         <v>28</v>
       </c>
@@ -1789,7 +1789,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="10" t="s">
         <v>34</v>
       </c>
@@ -1809,7 +1809,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="10" t="s">
         <v>34</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="10" t="s">
         <v>34</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="10" t="s">
         <v>34</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="10" t="s">
         <v>35</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="10" t="s">
         <v>35</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="10" t="s">
         <v>35</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="10" t="s">
         <v>35</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="10" t="s">
         <v>34</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="10" t="s">
         <v>34</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="10" t="s">
         <v>34</v>
       </c>
@@ -1999,7 +1999,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="10" t="s">
         <v>34</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="10" t="s">
         <v>34</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="10" t="s">
         <v>34</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="10" t="s">
         <v>34</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="10" t="s">
         <v>34</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="10" t="s">
         <v>35</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="10" t="s">
         <v>35</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="10" t="s">
         <v>35</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="10" t="s">
         <v>35</v>
       </c>
@@ -2169,7 +2169,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="10" t="s">
         <v>35</v>
       </c>
@@ -2187,7 +2187,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" s="10" t="s">
         <v>35</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="10" t="s">
         <v>35</v>
       </c>
@@ -2227,7 +2227,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" s="10" t="s">
         <v>35</v>
       </c>
@@ -2254,14 +2254,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59309159-8C26-48BD-9A2A-F4FDF67C921D}">
   <dimension ref="A1:D173"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="1" max="1" width="14.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="D2" s="6"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="D3" s="6"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="D4" s="6"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="D6" s="6"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -2344,7 +2344,7 @@
       </c>
       <c r="D7" s="6"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="D8" s="6"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -2368,7 +2368,7 @@
       </c>
       <c r="D9" s="6"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="D10" s="6"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="D11" s="6"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="D12" s="6"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="D13" s="6"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="D14" s="6"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="D15" s="6"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="D16" s="6"/>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="D17" s="6"/>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D18" s="6"/>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -2488,7 +2488,7 @@
       </c>
       <c r="D19" s="6"/>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="D20" s="6"/>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="D21" s="6"/>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="D22" s="6"/>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="D23" s="6"/>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>7</v>
       </c>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="D24" s="6"/>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>15</v>
       </c>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="D25" s="6"/>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>7</v>
       </c>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="D26" s="6"/>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -2584,7 +2584,7 @@
       </c>
       <c r="D27" s="6"/>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>7</v>
       </c>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="D28" s="6"/>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D29" s="6"/>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>7</v>
       </c>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="D30" s="6"/>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="D31" s="6"/>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>7</v>
       </c>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="D32" s="6"/>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>15</v>
       </c>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="D33" s="6"/>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>7</v>
       </c>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="D34" s="6"/>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>15</v>
       </c>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="D35" s="6"/>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>7</v>
       </c>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="D36" s="6"/>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>15</v>
       </c>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D37" s="6"/>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>7</v>
       </c>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="D38" s="6"/>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>15</v>
       </c>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="D39" s="6"/>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>7</v>
       </c>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="D40" s="6"/>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>15</v>
       </c>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="D41" s="6"/>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>7</v>
       </c>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="D42" s="6"/>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>15</v>
       </c>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="D43" s="6"/>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>7</v>
       </c>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="D44" s="6"/>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>15</v>
       </c>
@@ -2800,7 +2800,7 @@
       </c>
       <c r="D45" s="6"/>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>7</v>
       </c>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="D46" s="6"/>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>15</v>
       </c>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="D47" s="6"/>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>7</v>
       </c>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="D48" s="6"/>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>15</v>
       </c>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="D49" s="6"/>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>7</v>
       </c>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="D50" s="6"/>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>15</v>
       </c>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="D51" s="6"/>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>7</v>
       </c>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="D52" s="6"/>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>15</v>
       </c>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="D53" s="6"/>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>7</v>
       </c>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="D54" s="6"/>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>15</v>
       </c>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="D55" s="6"/>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>7</v>
       </c>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D56" s="6"/>
     </row>
-    <row r="57" spans="1:4">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>15</v>
       </c>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="D57" s="6"/>
     </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>7</v>
       </c>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="D58" s="6"/>
     </row>
-    <row r="59" spans="1:4">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>15</v>
       </c>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="D59" s="6"/>
     </row>
-    <row r="60" spans="1:4">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>7</v>
       </c>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="D60" s="6"/>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>15</v>
       </c>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D61" s="6"/>
     </row>
-    <row r="62" spans="1:4">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="D62" s="6"/>
     </row>
-    <row r="63" spans="1:4">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>15</v>
       </c>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="D63" s="6"/>
     </row>
-    <row r="64" spans="1:4">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>7</v>
       </c>
@@ -3028,7 +3028,7 @@
       </c>
       <c r="D64" s="6"/>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>15</v>
       </c>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="D65" s="6"/>
     </row>
-    <row r="66" spans="1:4">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>7</v>
       </c>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="D66" s="6"/>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>15</v>
       </c>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D67" s="6"/>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>7</v>
       </c>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="D68" s="6"/>
     </row>
-    <row r="69" spans="1:4">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>15</v>
       </c>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="D69" s="6"/>
     </row>
-    <row r="70" spans="1:4">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>7</v>
       </c>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="D70" s="6"/>
     </row>
-    <row r="71" spans="1:4">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>15</v>
       </c>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="D71" s="6"/>
     </row>
-    <row r="72" spans="1:4">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>7</v>
       </c>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="D72" s="6"/>
     </row>
-    <row r="73" spans="1:4">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>15</v>
       </c>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="D73" s="6"/>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>7</v>
       </c>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="D74" s="6"/>
     </row>
-    <row r="75" spans="1:4">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>15</v>
       </c>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="D75" s="6"/>
     </row>
-    <row r="76" spans="1:4">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>7</v>
       </c>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="D76" s="6"/>
     </row>
-    <row r="77" spans="1:4">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>15</v>
       </c>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="D77" s="6"/>
     </row>
-    <row r="78" spans="1:4">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>7</v>
       </c>
@@ -3195,21 +3195,21 @@
         <v>59.488</v>
       </c>
     </row>
-    <row r="161" spans="2:3">
+    <row r="161" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
     </row>
-    <row r="162" spans="2:3">
+    <row r="162" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
     </row>
-    <row r="163" spans="2:3">
+    <row r="163" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B163" s="1"/>
     </row>
-    <row r="169" spans="2:3">
+    <row r="169" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B169" s="1"/>
     </row>
-    <row r="173" spans="2:3">
+    <row r="173" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B173" s="1"/>
     </row>
   </sheetData>
@@ -3221,15 +3221,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4B4D9E9-39BD-4101-B02D-2FB2C2CEDBBB}">
   <dimension ref="A1:D183"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="14.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" customWidth="1"/>
+    <col min="4" max="4" width="17.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>24.591900000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="D3" s="6"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>25.0519</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>26.069900000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>26.146900000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>26.2469</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>26.514900000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -3329,7 +3329,7 @@
         <v>26.8369</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -3340,7 +3340,7 @@
         <v>27.161900000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>27.297900000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -3362,7 +3362,7 @@
         <v>27.315900000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>28.000900000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>28.303900000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -3395,7 +3395,7 @@
         <v>28.398900000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -3406,7 +3406,7 @@
         <v>28.600900000000003</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -3417,7 +3417,7 @@
         <v>28.943900000000003</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>29.068900000000003</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -3439,7 +3439,7 @@
         <v>29.2149</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>29.283900000000003</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -3461,7 +3461,7 @@
         <v>30.538900000000002</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -3472,7 +3472,7 @@
         <v>31.430900000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -3483,7 +3483,7 @@
         <v>31.5319</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>7</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>31.597900000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>15</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>32.430900000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>7</v>
       </c>
@@ -3516,7 +3516,7 @@
         <v>32.658900000000003</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -3527,7 +3527,7 @@
         <v>32.855899999999998</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>7</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>33.192900000000002</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -3549,7 +3549,7 @@
         <v>33.407899999999998</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>7</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>33.504899999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v>33.6479</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>7</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>33.709900000000005</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>15</v>
       </c>
@@ -3593,7 +3593,7 @@
         <v>34.334900000000005</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>7</v>
       </c>
@@ -3604,7 +3604,7 @@
         <v>34.435900000000004</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>15</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>34.611899999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>7</v>
       </c>
@@ -3626,7 +3626,7 @@
         <v>34.681899999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>15</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>34.995899999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>7</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>35.672899999999998</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>15</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>35.815899999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>7</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>36.042900000000003</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>15</v>
       </c>
@@ -3681,7 +3681,7 @@
         <v>36.134900000000002</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>7</v>
       </c>
@@ -3692,7 +3692,7 @@
         <v>36.178899999999999</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>15</v>
       </c>
@@ -3703,7 +3703,7 @@
         <v>36.243900000000004</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>7</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>36.300899999999999</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>15</v>
       </c>
@@ -3725,7 +3725,7 @@
         <v>36.950900000000004</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>7</v>
       </c>
@@ -3736,7 +3736,7 @@
         <v>37.829900000000002</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>15</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>38.064900000000002</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>7</v>
       </c>
@@ -3758,7 +3758,7 @@
         <v>38.128900000000002</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>15</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>38.429900000000004</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>7</v>
       </c>
@@ -3780,7 +3780,7 @@
         <v>40.692900000000002</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>15</v>
       </c>
@@ -3791,7 +3791,7 @@
         <v>41.240900000000003</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>7</v>
       </c>
@@ -3802,7 +3802,7 @@
         <v>42.0169</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>15</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>43.549900000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>7</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>43.919899999999998</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>15</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>44.273900000000005</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>7</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>44.483899999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>15</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>44.849899999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>7</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>45.154900000000005</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>15</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>46.274900000000002</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>7</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>46.297899999999998</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>15</v>
       </c>
@@ -3901,7 +3901,7 @@
         <v>47.099899999999998</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>47.313900000000004</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>15</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>47.431899999999999</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>7</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>47.832900000000002</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>15</v>
       </c>
@@ -3945,7 +3945,7 @@
         <v>48.499900000000004</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>7</v>
       </c>
@@ -3956,7 +3956,7 @@
         <v>48.749900000000004</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>15</v>
       </c>
@@ -3967,7 +3967,7 @@
         <v>49.4129</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>7</v>
       </c>
@@ -3978,7 +3978,7 @@
         <v>50.334900000000005</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>15</v>
       </c>
@@ -3989,7 +3989,7 @@
         <v>50.4709</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>7</v>
       </c>
@@ -4000,7 +4000,7 @@
         <v>50.8949</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>15</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>51.0289</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>7</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>51.5199</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>15</v>
       </c>
@@ -4033,7 +4033,7 @@
         <v>52.050899999999999</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>7</v>
       </c>
@@ -4044,7 +4044,7 @@
         <v>52.939900000000002</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>15</v>
       </c>
@@ -4055,7 +4055,7 @@
         <v>53.902900000000002</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>7</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>53.953900000000004</v>
       </c>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>15</v>
       </c>
@@ -4077,7 +4077,7 @@
         <v>56.873899999999999</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>7</v>
       </c>
@@ -4088,7 +4088,7 @@
         <v>57.110900000000001</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>15</v>
       </c>
@@ -4099,7 +4099,7 @@
         <v>57.899900000000002</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>7</v>
       </c>
@@ -4110,7 +4110,7 @@
         <v>58.414900000000003</v>
       </c>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>15</v>
       </c>
@@ -4121,7 +4121,7 @@
         <v>58.977899999999998</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>7</v>
       </c>
@@ -4132,21 +4132,21 @@
         <v>59.48</v>
       </c>
     </row>
-    <row r="171" spans="2:3">
+    <row r="171" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
     </row>
-    <row r="172" spans="2:3">
+    <row r="172" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
     </row>
-    <row r="173" spans="2:3">
+    <row r="173" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B173" s="1"/>
     </row>
-    <row r="179" spans="2:2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B179" s="1"/>
     </row>
-    <row r="183" spans="2:2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B183" s="1"/>
     </row>
   </sheetData>
@@ -4158,14 +4158,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A58A4A1B-2A66-4BD4-8004-4972898CE4F4}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.7265625" customWidth="1"/>
+    <col min="3" max="3" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>39</v>
       </c>
@@ -4176,7 +4176,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -4184,12 +4184,12 @@
         <v>24</v>
       </c>
       <c r="C2">
-        <v>28.309899999999999</v>
+        <v>28.300899999999999</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -4202,7 +4202,7 @@
       <c r="D3" s="6"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -4215,7 +4215,7 @@
       <c r="D4" s="6"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -4228,7 +4228,7 @@
       <c r="D5" s="6"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -4241,7 +4241,7 @@
       <c r="D6" s="6"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -4261,25 +4261,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Descriptive_x0020_Name xmlns="c32bb4e5-d30f-47c7-b40d-8e40c9a47274" xsi:nil="true"/>
-    <IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/>
-    <_dlc_DocId xmlns="a4282dde-c91e-40c5-9bfe-d2af68f8b118">D3WV7AQZNZZ4-1479232743-7688281</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="a4282dde-c91e-40c5-9bfe-d2af68f8b118">
-      <Url>https://mtrchk.sharepoint.com/sites/doms_imd3/_layouts/15/DocIdRedir.aspx?ID=D3WV7AQZNZZ4-1479232743-7688281</Url>
-      <Description>D3WV7AQZNZZ4-1479232743-7688281</Description>
-    </_dlc_DocIdUrl>
-    <j5297b21f81e4c988d0459bda67ca59f xmlns="f57c62ac-5b60-40b7-9460-0473ac1a050a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j5297b21f81e4c988d0459bda67ca59f>
-    <link xmlns="f57c62ac-5b60-40b7-9460-0473ac1a050a">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </link>
-    <TaxCatchAll xmlns="a4282dde-c91e-40c5-9bfe-d2af68f8b118" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4508,12 +4495,25 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Descriptive_x0020_Name xmlns="c32bb4e5-d30f-47c7-b40d-8e40c9a47274" xsi:nil="true"/>
+    <IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/>
+    <_dlc_DocId xmlns="a4282dde-c91e-40c5-9bfe-d2af68f8b118">D3WV7AQZNZZ4-1479232743-7688281</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="a4282dde-c91e-40c5-9bfe-d2af68f8b118">
+      <Url>https://mtrchk.sharepoint.com/sites/doms_imd3/_layouts/15/DocIdRedir.aspx?ID=D3WV7AQZNZZ4-1479232743-7688281</Url>
+      <Description>D3WV7AQZNZZ4-1479232743-7688281</Description>
+    </_dlc_DocIdUrl>
+    <j5297b21f81e4c988d0459bda67ca59f xmlns="f57c62ac-5b60-40b7-9460-0473ac1a050a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j5297b21f81e4c988d0459bda67ca59f>
+    <link xmlns="f57c62ac-5b60-40b7-9460-0473ac1a050a">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </link>
+    <TaxCatchAll xmlns="a4282dde-c91e-40c5-9bfe-d2af68f8b118" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4567,17 +4567,51 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEE95442-7288-4EE9-BCC4-F58766902565}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{535E1E83-88F3-49B8-AD34-B800272C6BCD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{590E65BA-16C0-44FA-A032-559EB6A58F9A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{590E65BA-16C0-44FA-A032-559EB6A58F9A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c32bb4e5-d30f-47c7-b40d-8e40c9a47274"/>
+    <ds:schemaRef ds:uri="f57c62ac-5b60-40b7-9460-0473ac1a050a"/>
+    <ds:schemaRef ds:uri="a4282dde-c91e-40c5-9bfe-d2af68f8b118"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{535E1E83-88F3-49B8-AD34-B800272C6BCD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEE95442-7288-4EE9-BCC4-F58766902565}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c32bb4e5-d30f-47c7-b40d-8e40c9a47274"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
+    <ds:schemaRef ds:uri="a4282dde-c91e-40c5-9bfe-d2af68f8b118"/>
+    <ds:schemaRef ds:uri="f57c62ac-5b60-40b7-9460-0473ac1a050a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{417ACB90-4253-44FF-A201-2B52C95D02C8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{417ACB90-4253-44FF-A201-2B52C95D02C8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>